<commit_message>
Add Intro to AI lecture 1 notes and Anki tables, and record Anki note IDs on DE and ProbStat cards.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/DifferentialEquations/notes/anki_cards/DIFF Lection 1 - введение_anki_cards.xlsx
+++ b/DifferentialEquations/notes/anki_cards/DIFF Lection 1 - введение_anki_cards.xlsx
@@ -504,7 +504,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>1788372005875</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -547,7 +549,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>1788372005877</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -590,7 +594,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>1788372005878</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -633,7 +639,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>1788372005879</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -676,7 +684,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="n">
+        <v>1788372005880</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -719,7 +729,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>1788372005881</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -762,7 +774,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>1788372005882</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -805,7 +819,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>1788372005883</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -848,7 +864,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>1788372005884</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -891,7 +909,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>1788372005885</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -934,7 +954,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>1788372005886</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -977,7 +999,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>1788372005887</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1020,7 +1044,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>1788372005888</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1063,7 +1089,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>1788372005889</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1106,7 +1134,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>1788372005890</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1149,7 +1179,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>1788372005891</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1192,7 +1224,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>1788372005892</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1235,7 +1269,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>1788372005893</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1278,7 +1314,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>1788372005894</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1321,7 +1359,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>1788372005895</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1364,7 +1404,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>1788372005896</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1407,7 +1449,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>1788372005897</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1450,7 +1494,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>1788372005898</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1493,7 +1539,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="n">
+        <v>1788372005899</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1536,7 +1584,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
+      <c r="I26" t="n">
+        <v>1788372005900</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1579,7 +1629,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
+      <c r="I27" t="n">
+        <v>1788372005901</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1622,7 +1674,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
+      <c r="I28" t="n">
+        <v>1788372005902</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1665,7 +1719,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
+      <c r="I29" t="n">
+        <v>1788372005903</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1708,7 +1764,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
+      <c r="I30" t="n">
+        <v>1788372005904</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1751,7 +1809,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="n">
+        <v>1788372005905</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1794,7 +1854,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="n">
+        <v>1788372005906</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1837,7 +1899,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" t="n">
+        <v>1788372005907</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1880,7 +1944,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" t="n">
+        <v>1788372005908</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1923,7 +1989,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
+      <c r="I35" t="n">
+        <v>1788372005909</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1966,7 +2034,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
+      <c r="I36" t="n">
+        <v>1788372005910</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2009,7 +2079,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="n">
+        <v>1788372005911</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2052,7 +2124,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
+      <c r="I38" t="n">
+        <v>1788372051430</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2095,7 +2169,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="n">
+        <v>1788372051431</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2138,7 +2214,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="n">
+        <v>1788372051432</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2181,7 +2259,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
+      <c r="I41" t="n">
+        <v>1788372051433</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2224,7 +2304,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
+      <c r="I42" t="n">
+        <v>1788372051434</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2267,7 +2349,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
+      <c r="I43" t="n">
+        <v>1788372051435</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2310,7 +2394,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
+      <c r="I44" t="n">
+        <v>1788372051436</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2353,7 +2439,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
+      <c r="I45" t="n">
+        <v>1788372051437</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2396,7 +2484,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
+      <c r="I46" t="n">
+        <v>1788372051438</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2439,7 +2529,9 @@
           <t>Inno_2course_1semester::Differential Equations</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
+      <c r="I47" t="n">
+        <v>1788372051439</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>